<commit_message>
Update bank interest rate report
</commit_message>
<xml_diff>
--- a/output/interest_rate_report.xlsx
+++ b/output/interest_rate_report.xlsx
@@ -2250,7 +2250,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>https://images.merolagani.com//content/bigyapan/f4ac68d3-5980-4c7e-9896-932b1c160de4.gif</t>
+          <t>https://images.merolagani.com//content/bigyapan/35bf8124-cfc0-4314-a1b3-c251ad1eb605.gif</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">

</xml_diff>